<commit_message>
chore: update and sync node_modules and android build artifacts
</commit_message>
<xml_diff>
--- a/project docs/FameU_Master_Project_Sheet.xlsx
+++ b/project docs/FameU_Master_Project_Sheet.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chandanmallik/projects/Fameu/project docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED8BE487-91C2-F54C-AF75-710A2EF020D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E5B211-8486-1E4A-AFD9-CECAF2DF6187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3980" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{520AB9B4-5B8B-D74E-B4B5-658DA24739EE}"/>
   </bookViews>
   <sheets>
     <sheet name="FameU_Master_Project_Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FameU_Master_Project_Sheet!$A$1:$F$47</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1415,6 +1418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB06232C-E172-3642-ABCF-5ABD29DEBAF4}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1571,7 +1575,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1592,7 +1596,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1613,7 +1617,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1634,7 +1638,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1655,7 +1659,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1676,7 +1680,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1697,7 +1701,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1718,7 +1722,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1739,7 +1743,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1760,7 +1764,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1781,7 +1785,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1802,7 +1806,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2033,7 +2037,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -2054,7 +2058,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -2075,7 +2079,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -2096,7 +2100,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -2117,7 +2121,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -2138,7 +2142,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -2159,7 +2163,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -2180,7 +2184,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -2201,7 +2205,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -2222,7 +2226,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -2243,7 +2247,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -2264,7 +2268,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -2285,7 +2289,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -2306,7 +2310,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -2327,7 +2331,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -2348,7 +2352,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -2369,7 +2373,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -2390,7 +2394,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -2412,6 +2416,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F47" xr:uid="{BB06232C-E172-3642-ABCF-5ABD29DEBAF4}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Both Apps"/>
+        <filter val="Hiring App"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: update Android application IDs, adjust project strings, and add new Privacy Policy page to website
</commit_message>
<xml_diff>
--- a/project docs/FameU_Master_Project_Sheet.xlsx
+++ b/project docs/FameU_Master_Project_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chandanmallik/projects/Fameu/project docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E5B211-8486-1E4A-AFD9-CECAF2DF6187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E624B77-C764-454E-9A4A-F29E0E2F8013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3980" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{520AB9B4-5B8B-D74E-B4B5-658DA24739EE}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{520AB9B4-5B8B-D74E-B4B5-658DA24739EE}"/>
   </bookViews>
   <sheets>
     <sheet name="FameU_Master_Project_Sheet" sheetId="1" r:id="rId1"/>
@@ -1418,7 +1418,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB06232C-E172-3642-ABCF-5ABD29DEBAF4}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1575,7 +1574,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1596,7 +1595,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1617,7 +1616,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1638,7 +1637,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1659,7 +1658,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1680,7 +1679,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1701,7 +1700,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1722,7 +1721,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1743,7 +1742,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1764,7 +1763,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1785,7 +1784,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1806,7 +1805,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2037,7 +2036,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -2058,7 +2057,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -2079,7 +2078,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -2100,7 +2099,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -2121,7 +2120,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -2142,7 +2141,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -2163,7 +2162,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -2184,7 +2183,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -2205,7 +2204,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -2226,7 +2225,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -2247,7 +2246,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -2268,7 +2267,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -2289,7 +2288,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -2310,7 +2309,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -2331,7 +2330,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -2352,7 +2351,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -2373,7 +2372,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -2394,7 +2393,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -2416,14 +2415,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F47" xr:uid="{BB06232C-E172-3642-ABCF-5ABD29DEBAF4}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Both Apps"/>
-        <filter val="Hiring App"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F47" xr:uid="{BB06232C-E172-3642-ABCF-5ABD29DEBAF4}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>